<commit_message>
feat: implement loaders for storefront navigation and enhance UI feedback
- Added a page loader and busy indicators for buttons to improve user experience during navigation and actions.
- Introduced `Loader` and `LoaderMark` components for consistent loading visuals.
- Updated CSS for loaders to ensure they respect user preferences for reduced motion.
- Integrated loading states into various components including buttons in account management, checkout, and product actions.
- Enhanced navigation experience with `NavigationLoader` to show loading indicators during page transitions.
- Updated documentation to reflect changes in testing and coverage for new loader functionality.
</commit_message>
<xml_diff>
--- a/docs/qa/TenantEcom-test-cases.xlsx
+++ b/docs/qa/TenantEcom-test-cases.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Vendor CMS'!$A$1:$U$198</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Super Admin'!$A$1:$U$106</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'End-to-End Workflows'!$A$1:$U$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'End-to-End Workflows'!$A$1:$U$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Defect Log'!$A$1:$M$204</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-13 from docs/qa/tools. Figures recalculate as Status cells change.</t>
+          <t>Generated 2026-10-14 from docs/qa/tools. Figures recalculate as Status cells change.</t>
         </is>
       </c>
     </row>
@@ -31493,7 +31493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U53"/>
+  <dimension ref="A1:U54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -36521,9 +36521,102 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>E2E-18-008</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>End-to-End</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>E2E-18 · Storefront chrome and search (shop experience)</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Loaders</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>Page loader and busy buttons</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>Moving between pages and waiting on a button both show the store’s loader, and a missing page still answers 404.</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>Store selling; Chrome DevTools → Network → Slow 4G for the slow steps</t>
+        </is>
+      </c>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>Any product; pincode 560001; /products/no-such-product</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>1. Click a category, then a product (Slow 4G)
+2. Search from the header and press Enter
+3. Add to cart, Buy now and Check the pincode on a product
+4. Place an order (COD)
+5. Turn animations off in the system and repeat one step
+6. Open /products/no-such-product directly
+7. Verify the expected result.</t>
+        </is>
+      </c>
+      <c r="J54" s="11" t="inlineStr">
+        <is>
+          <t>A thin bar in the store colour at the top at once; after about half a second the house with a dot circling it and "Loading…" in the middle, gone when the page arrives (quick pages show neither); only the pressed button shows a small ring with its words; the order page loads under the loader; with animations off the ring and dot fade instead of turning; the missing product answers 404 (a moved one still redirects).</t>
+        </is>
+      </c>
+      <c r="K54" s="11" t="inlineStr"/>
+      <c r="L54" s="11" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="M54" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N54" s="11" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="O54" s="11" t="inlineStr"/>
+      <c r="P54" s="11" t="inlineStr"/>
+      <c r="Q54" s="11" t="inlineStr"/>
+      <c r="R54" s="11" t="inlineStr"/>
+      <c r="S54" s="11" t="inlineStr">
+        <is>
+          <t>Shopper</t>
+        </is>
+      </c>
+      <c r="T54" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U54" s="11" t="inlineStr">
+        <is>
+          <t>docs/qa/regression/e2e/E2E-18-storefront.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U53"/>
-  <conditionalFormatting sqref="L2:L253">
+  <autoFilter ref="A1:U54"/>
+  <conditionalFormatting sqref="L2:L254">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Pass"</formula>
     </cfRule>
@@ -36540,25 +36633,25 @@
       <formula>"Not Applicable"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M253">
+  <conditionalFormatting sqref="M2:M254">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
       <formula>"Critical"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="L2:L253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+    <dataValidation sqref="L2:L254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"Not Run,Pass,Fail,Blocked,Not Applicable"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+    <dataValidation sqref="M2:M254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+    <dataValidation sqref="N2:N254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"Functional,Regression,Negative,Validation,Boundary,Integration,UI/UX,Security/Permissions,Data persistence,Accessibility"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+    <dataValidation sqref="B2:B254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"Super Admin,Vendor CMS,End-to-End"</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T253" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
+    <dataValidation sqref="T2:T254" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a value from the list" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>